<commit_message>
fix: normalize direct barging
</commit_message>
<xml_diff>
--- a/imports/templates/geology_ore_import_template.xlsx
+++ b/imports/templates/geology_ore_import_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Documents/template-import/alpha-mines/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Project/python/mines-smart/imports/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D4BC90-C568-F847-8593-CDD3316EF981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D11132D-A590-7A4D-A91E-421A911995C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="35980" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-4740" yWindow="780" windowWidth="35980" windowHeight="20880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_ore" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="64">
   <si>
     <t>Kolom wajib:</t>
   </si>
@@ -57,15 +57,6 @@
     <t>iup_code</t>
   </si>
   <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>LIS</t>
-  </si>
-  <si>
-    <t>SAS</t>
-  </si>
-  <si>
     <t>- iup_code (wajib, unik)</t>
   </si>
   <si>
@@ -75,30 +66,9 @@
     <t>- Untuk kolom wajib isi, dengan warna kuning pada nama header kolom</t>
   </si>
   <si>
-    <t>sublot_close</t>
-  </si>
-  <si>
     <t>SL_01</t>
   </si>
   <si>
-    <t>SL_02</t>
-  </si>
-  <si>
-    <t>SL_03</t>
-  </si>
-  <si>
-    <t>SL_04</t>
-  </si>
-  <si>
-    <t>SL_05</t>
-  </si>
-  <si>
-    <t>SL_06</t>
-  </si>
-  <si>
-    <t>SL_07</t>
-  </si>
-  <si>
     <t>1) Isi sheet 'sale_code' mulai baris 2.</t>
   </si>
   <si>
@@ -229,17 +199,45 @@
   </si>
   <si>
     <t>Dumping A</t>
+  </si>
+  <si>
+    <t>pit_dome</t>
+  </si>
+  <si>
+    <t>direct</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Direct Barging</t>
+  </si>
+  <si>
+    <t>KWS-00135</t>
+  </si>
+  <si>
+    <t>Trial direct</t>
+  </si>
+  <si>
+    <t>LGS</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="h:mm;@"/>
+    <numFmt numFmtId="166" formatCode="[$-409]d\-mmm\-yy;@"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -272,25 +270,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -343,6 +322,12 @@
       <charset val="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -377,8 +362,8 @@
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="26">
@@ -386,9 +371,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -396,46 +378,55 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -741,283 +732,450 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="8.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" style="15" customWidth="1"/>
-    <col min="5" max="5" width="20.5" style="15" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" style="15" customWidth="1"/>
-    <col min="7" max="7" width="9" style="1" customWidth="1"/>
-    <col min="8" max="8" width="11.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.83203125" style="10" customWidth="1"/>
+    <col min="5" max="5" width="12.1640625" style="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" style="10" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1640625" style="1" customWidth="1"/>
     <col min="9" max="9" width="9.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" style="15" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10" style="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1640625" style="1" customWidth="1"/>
     <col min="12" max="12" width="11.83203125" customWidth="1"/>
     <col min="13" max="13" width="10.1640625" customWidth="1"/>
-    <col min="14" max="14" width="13.5" style="15" customWidth="1"/>
+    <col min="14" max="14" width="13.5" style="10" customWidth="1"/>
     <col min="15" max="15" width="11.6640625" customWidth="1"/>
-    <col min="16" max="16" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12.6640625" customWidth="1"/>
-    <col min="19" max="19" width="8.1640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="12" customWidth="1"/>
+    <col min="18" max="18" width="11.83203125" customWidth="1"/>
+    <col min="19" max="19" width="6.83203125" customWidth="1"/>
+    <col min="20" max="20" width="10.33203125" customWidth="1"/>
+    <col min="21" max="21" width="10.5" customWidth="1"/>
+    <col min="22" max="22" width="12.1640625" customWidth="1"/>
+    <col min="23" max="23" width="11.5" customWidth="1"/>
+    <col min="24" max="24" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="L1" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="N1" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="P1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="D1" s="12" t="s">
+      <c r="Q1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="R1" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="S1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="16" t="s">
+      <c r="T1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="U1" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="12" t="s">
+      <c r="V1" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="W1" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="X1" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="Y1" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="14">
+        <v>45800</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G2" s="17"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" s="22"/>
+      <c r="L2" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="M2" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="N2" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="O2" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="25">
+        <v>8</v>
+      </c>
+      <c r="R2" t="s">
+        <v>45</v>
+      </c>
+      <c r="S2">
+        <v>3</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2" t="s">
+        <v>46</v>
+      </c>
+      <c r="W2" t="s">
+        <v>47</v>
+      </c>
+      <c r="X2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y2" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="14">
+        <v>45801</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="17"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="22"/>
+      <c r="L3" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="N3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="O3" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="P3" s="1">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="25">
+        <v>5</v>
+      </c>
+      <c r="R3" t="s">
+        <v>45</v>
+      </c>
+      <c r="S3">
+        <v>2</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3" t="s">
+        <v>46</v>
+      </c>
+      <c r="W3" t="s">
+        <v>47</v>
+      </c>
+      <c r="X3" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="14">
+        <v>45801</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" s="17"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="22"/>
+      <c r="L4" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="P4" s="1">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="25">
+        <v>5</v>
+      </c>
+      <c r="R4" t="s">
+        <v>45</v>
+      </c>
+      <c r="S4">
+        <v>6</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4" t="s">
+        <v>46</v>
+      </c>
+      <c r="W4" t="s">
+        <v>47</v>
+      </c>
+      <c r="X4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="21">
+        <v>46196</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="17"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="22"/>
+      <c r="L5" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="K1" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="M1" s="14" t="s">
+      <c r="O5" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q5" s="25">
+        <v>5</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="S5">
+        <v>2</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5" t="s">
+        <v>46</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="W5" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="X5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="21">
+        <v>46196</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="14" t="s">
+      <c r="E6" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="17"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="22"/>
+      <c r="L6" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="M6" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="P1" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q1" s="14" t="s">
+      <c r="N6" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="O6" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q6" s="25">
+        <v>5</v>
+      </c>
+      <c r="R6" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="R1" s="14" t="s">
+      <c r="S6">
+        <v>2</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6" t="s">
         <v>46</v>
       </c>
-      <c r="S1" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="T1" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="U1" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="V1" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="W1" s="18" t="s">
+      <c r="V6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="W6" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="19">
-        <v>45800</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="F2" s="22"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="J2" s="24"/>
-      <c r="K2" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="L2" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="M2" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
-        <v>8</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>55</v>
-      </c>
-      <c r="R2">
-        <v>3</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2" t="s">
-        <v>56</v>
-      </c>
-      <c r="V2" t="s">
-        <v>57</v>
-      </c>
-      <c r="W2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B3" s="19">
-        <v>45801</v>
-      </c>
-      <c r="C3" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" s="22"/>
-      <c r="G3" s="23"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="24"/>
-      <c r="K3" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="L3" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="M3" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="N3" s="24" t="s">
+      <c r="X6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y6" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="O3">
-        <v>2</v>
-      </c>
-      <c r="P3">
-        <v>5</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>55</v>
-      </c>
-      <c r="R3">
-        <v>2</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3" t="s">
-        <v>56</v>
-      </c>
-      <c r="V3" t="s">
-        <v>57</v>
-      </c>
-      <c r="W3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="19">
-        <v>45801</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="F4" s="22"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="J4" s="24"/>
-      <c r="K4" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="L4" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="M4" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="N4" s="24" t="s">
-        <v>63</v>
-      </c>
-      <c r="O4">
-        <v>3</v>
-      </c>
-      <c r="P4">
-        <v>5</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>55</v>
-      </c>
-      <c r="R4">
-        <v>6</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4" t="s">
-        <v>56</v>
-      </c>
-      <c r="V4" t="s">
-        <v>57</v>
-      </c>
-      <c r="W4" t="s">
-        <v>53</v>
-      </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
@@ -1025,163 +1183,114 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="90" customWidth="1"/>
     <col min="2" max="2" width="7.33203125" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" customWidth="1"/>
-    <col min="4" max="4" width="5.1640625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.6640625" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1" s="13" t="s">
+    <row r="1" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="4"/>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="13" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6"/>
+    </row>
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="5"/>
-    </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="7"/>
-      <c r="C2" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+    </row>
+    <row r="16" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
+    </row>
+    <row r="18" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="9"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="9" t="s">
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="7"/>
-    </row>
-    <row r="18" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
   </sheetData>
-  <phoneticPr fontId="10" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>